<commit_message>
Auto-opdater EPGOAL 2026-10-05 23:08:44
</commit_message>
<xml_diff>
--- a/data/channel_priority_v2.xlsx
+++ b/data/channel_priority_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634C0100-6576-4A3E-A797-C71D9B6B8364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B13CE5C-C7E5-44EA-8D70-5337A19CB60D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kanal-prioritering v2" sheetId="1" r:id="rId1"/>
@@ -1145,12 +1145,6 @@
     <t>tlc.dk</t>
   </si>
   <si>
-    <t>tv3.dk</t>
-  </si>
-  <si>
-    <t>tv3plus.dk</t>
-  </si>
-  <si>
     <t>bbcworldnews.uk</t>
   </si>
   <si>
@@ -1179,6 +1173,12 @@
   </si>
   <si>
     <t>viasatultra.dk</t>
+  </si>
+  <si>
+    <t>news.dk</t>
+  </si>
+  <si>
+    <t>tv3.puls.dk</t>
   </si>
 </sst>
 </file>
@@ -1553,20 +1553,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K62"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
     <col min="6" max="6" width="55" customWidth="1"/>
-    <col min="7" max="7" width="23.7265625" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" customWidth="1"/>
     <col min="8" max="9" width="44" customWidth="1"/>
     <col min="10" max="10" width="68" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
@@ -1699,10 +1699,10 @@
         <v>29</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>41</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>45</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>52</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>61</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>68</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>75</v>
       </c>
@@ -1979,10 +1979,10 @@
         <v>81</v>
       </c>
       <c r="K13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>82</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>87</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>92</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>99</v>
       </c>
@@ -2108,10 +2108,10 @@
         <v>103</v>
       </c>
       <c r="K17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>104</v>
       </c>
@@ -2141,10 +2141,10 @@
         <v>108</v>
       </c>
       <c r="K18" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>109</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>114</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>120</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>127</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>134</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>141</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>145</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>147</v>
       </c>
@@ -2394,7 +2394,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>154</v>
       </c>
@@ -2427,7 +2427,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>161</v>
       </c>
@@ -2460,7 +2460,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>168</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>171</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>176</v>
       </c>
@@ -2545,10 +2545,10 @@
         <v>180</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>181</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>183</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>185</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>190</v>
       </c>
@@ -2659,7 +2659,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>196</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>200</v>
       </c>
@@ -2707,10 +2707,10 @@
         <v>204</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>205</v>
       </c>
@@ -2734,10 +2734,10 @@
         <v>209</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>210</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>215</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>222</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>229</v>
       </c>
@@ -2858,10 +2858,10 @@
         <v>231</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>232</v>
       </c>
@@ -2891,10 +2891,10 @@
         <v>238</v>
       </c>
       <c r="K43" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>239</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>246</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>253</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>260</v>
       </c>
@@ -3026,7 +3026,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>267</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>274</v>
       </c>
@@ -3089,10 +3089,10 @@
         <v>280</v>
       </c>
       <c r="K49" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>281</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>288</v>
       </c>
@@ -3155,10 +3155,10 @@
         <v>293</v>
       </c>
       <c r="K51" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>294</v>
       </c>
@@ -3188,10 +3188,10 @@
         <v>298</v>
       </c>
       <c r="K52" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>299</v>
       </c>
@@ -3215,10 +3215,10 @@
         <v>301</v>
       </c>
       <c r="K53" s="4" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>302</v>
       </c>
@@ -3242,10 +3242,10 @@
         <v>306</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>307</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>312</v>
       </c>
@@ -3296,10 +3296,10 @@
         <v>316</v>
       </c>
       <c r="K56" s="4" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>317</v>
       </c>
@@ -3323,10 +3323,10 @@
         <v>321</v>
       </c>
       <c r="K57" s="4" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>322</v>
       </c>
@@ -3359,7 +3359,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>329</v>
       </c>
@@ -3383,10 +3383,10 @@
         <v>332</v>
       </c>
       <c r="K59" s="4" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>333</v>
       </c>
@@ -3419,7 +3419,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>339</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>343</v>
       </c>
@@ -3486,80 +3486,81 @@
   </sheetData>
   <autoFilter ref="A1:J62" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>360</v>
       </c>

</xml_diff>

<commit_message>
Auto-opdater EPGOAL 2026-10-06 08:51:11
</commit_message>
<xml_diff>
--- a/data/channel_priority_v2.xlsx
+++ b/data/channel_priority_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B13CE5C-C7E5-44EA-8D70-5337A19CB60D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52044216-73BB-484D-A490-F8327CADB12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2108,7 +2108,7 @@
         <v>103</v>
       </c>
       <c r="K17" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2141,7 +2141,7 @@
         <v>108</v>
       </c>
       <c r="K18" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">

</xml_diff>